<commit_message>
Actualiza Tarifas Ingeniería desde el portal
</commit_message>
<xml_diff>
--- a/ListaPreciosIngenieria.xlsx
+++ b/ListaPreciosIngenieria.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrador\Desktop\AplicativoIngenieria\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrador\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A665E4E-8840-485E-9622-80DB9A20D798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E93178E-7781-4E18-BF97-649B27A05AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="3" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="4" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
@@ -537,6 +538,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18E554C7-3182-47EC-9E89-F70C2BCAC2B4}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA56E166-B217-4475-A259-8C238D1A508F}">
   <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>